<commit_message>
EDW-33: extras entry could be read as a legitimate analog (same size, other DIN) - replaced before the first pipeline run
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmarks/attachment_intelligence/fixtures/files/f06.xlsx
+++ b/benchmarks/attachment_intelligence/fixtures/files/f06.xlsx
@@ -1128,12 +1128,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Гайка самоконтрящаяся M10 DIN 985</t>
+          <t xml:space="preserve">Гайка самоконтрящаяся M14 DIN 985</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">DIN985-M10</t>
+          <t xml:space="preserve">DIN985-M14</t>
         </is>
       </c>
       <c r="D41">
@@ -1145,10 +1145,10 @@
         </is>
       </c>
       <c r="F41">
-        <v>4.19</v>
+        <v>7.88</v>
       </c>
       <c r="G41">
-        <v>41.9</v>
+        <v>78.8</v>
       </c>
     </row>
     <row r="42">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">115 367,90</t>
+          <t xml:space="preserve">115 404,80</t>
         </is>
       </c>
     </row>

</xml_diff>